<commit_message>
Synthetic chain complete: Q2 2027 run, decided and published; second full pass clean; docs
All three quarters compare with 0 mismatches against their committed expectations on two consecutive
passes (the compare now runs each quarter undecided, with its own ledger records filtered out). Q2 2027
is decided and published (booked 1,106.0) and its build emitted the Q3 2027 input. Booked NAV, marks,
ownership, invested and cumulative realized tie across every boundary. Malformed variants now carry the
clean sidecar so each shows only its own defect, and a duplicated-funded-round variant is added.

HARDENING_REPORT.md carries every defect, the simulated decisions, the verification results, the policy
ambiguities and how to reproduce. CLAUDE.md and README describe --ledger-dir, the synthetic provider and
the dashboard's Workbook select.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0128YjwFzw9Zog7h4DXUWFdB
</commit_message>
<xml_diff>
--- a/data/quarters/synthetic/2027Q1/SYNTHETIC_portfolio_Q1_2027.xlsx
+++ b/data/quarters/synthetic/2027Q1/SYNTHETIC_portfolio_Q1_2027.xlsx
@@ -1730,7 +1730,7 @@
         <v>43895</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>44477</v>
+        <v>46245</v>
       </c>
       <c r="H17" s="13" t="n">
         <v>176.3</v>
@@ -9085,7 +9085,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>hc-valuation engine 0.1.0, policy 2026Q4-0.1, run b9e1bcc61c42</t>
+          <t>hc-valuation engine 0.1.0, policy 2026Q4-0.1, run df62f01d0864</t>
         </is>
       </c>
     </row>
@@ -9441,7 +9441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9541,6 +9541,18 @@
       <c r="B8" t="inlineStr">
         <is>
           <t>Entered the book in Q4 2026 from a New Investment row (M-014, X-918): fund, sector and stage are as that row named them, and the operating metrics (ARR, growth, margin, burn, cash, headcount) are blank because nothing is on file. Fill them before the next run.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Pellagrin</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>same-terms extension on 2026-08-11 is not price discovery; the staleness clock runs from 2021-10-08</t>
         </is>
       </c>
     </row>

</xml_diff>